<commit_message>
New Features & Bugfixes
- Fixed Biome to Biome banner display issues
- Added Wrench (misc)
- Added Arcane pool to arcane arrow
- Setup arcane archer custom attack style
- Built framework for gif-based attacks to display correctly in game(on a per-frame basis)
</commit_message>
<xml_diff>
--- a/Survivor Game.xlsx
+++ b/Survivor Game.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mtgra\Desktop\GameDev\SurvivorsLike\SurvivorsLike\SurvivorsLikeGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40CC9C69-AA0A-4926-AF5B-4112DD15A2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBAA7C8-408C-4CBC-A33A-3BAB3C145728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="358">
   <si>
     <t>Knight</t>
   </si>
@@ -1673,6 +1673,45 @@
   </si>
   <si>
     <t>Meta-Progression &amp; Hub Features</t>
+  </si>
+  <si>
+    <t>Psammomancer</t>
+  </si>
+  <si>
+    <t>Sand Shield</t>
+  </si>
+  <si>
+    <t>SandShield</t>
+  </si>
+  <si>
+    <t>Hivemaster</t>
+  </si>
+  <si>
+    <t>InsectSwarm</t>
+  </si>
+  <si>
+    <t>Insect Swarm</t>
+  </si>
+  <si>
+    <t>Geomancer</t>
+  </si>
+  <si>
+    <t>Aeromancer</t>
+  </si>
+  <si>
+    <t>Meteor Smash</t>
+  </si>
+  <si>
+    <t>MeteorSmash</t>
+  </si>
+  <si>
+    <t>Wind Storm</t>
+  </si>
+  <si>
+    <t>WindStorm</t>
+  </si>
+  <si>
+    <t>TimeManipulation</t>
   </si>
 </sst>
 </file>
@@ -2790,7 +2829,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0134B62F-E2D3-4D00-ACEE-B088AA598477}">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
@@ -2920,7 +2959,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="11" t="s">
         <v>201</v>
       </c>
       <c r="B12" t="s">
@@ -2931,7 +2970,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
+      <c r="A13" t="s">
         <v>202</v>
       </c>
       <c r="B13" t="s">
@@ -3092,11 +3131,11 @@
         <v>227</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>228</v>
+        <v>357</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="11" t="s">
         <v>229</v>
       </c>
       <c r="B28" t="s">
@@ -3107,7 +3146,7 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="11" t="s">
+      <c r="A29" t="s">
         <v>230</v>
       </c>
       <c r="B29" t="s">
@@ -3206,7 +3245,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="11" t="s">
         <v>172</v>
       </c>
       <c r="B38" t="s">
@@ -3228,7 +3267,7 @@
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="11" t="s">
         <v>173</v>
       </c>
       <c r="B40" t="s">
@@ -3250,7 +3289,7 @@
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="11" t="s">
+      <c r="A42" t="s">
         <v>174</v>
       </c>
       <c r="B42" t="s">
@@ -3283,7 +3322,7 @@
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="6" t="s">
+      <c r="A45" s="11" t="s">
         <v>178</v>
       </c>
       <c r="B45" t="s">
@@ -3302,6 +3341,50 @@
       </c>
       <c r="C46" t="s">
         <v>180</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update todo ideas for future modes
</commit_message>
<xml_diff>
--- a/Survivor Game.xlsx
+++ b/Survivor Game.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mtgra\Desktop\GameDev\SurvivorsLike\SurvivorsLike\SurvivorsLikeGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4646D8FD-42F2-427B-993D-DF10B4FADEB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B82FF5F-8F52-4EDC-8F69-0129BC2C6DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="304">
   <si>
     <t>Knight</t>
   </si>
@@ -808,864 +808,6 @@
     <t>OracleBeam</t>
   </si>
   <si>
-    <t>1. The Virus (Infection Mode)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">You don't collect weapons; you collect </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Pathogens</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Your "projectiles" are contagious. When you hit an enemy, they don't die instantly—they become infected and start damaging nearby enemies.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You have to manage the "Spread Rate" vs. "Lethality." If the virus kills too fast, it won't spread to the rest of the swarm. If it's too slow, you'll be overwhelmed.</t>
-    </r>
-  </si>
-  <si>
-    <t>2. Sigil Architect (Modular Rituals)</t>
-  </si>
-  <si>
-    <t>This mode turns the ground itself into your weapon.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You don't fire traditional projectiles. Instead, you drop "Connectors" and "Power Bricks" as you move.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> When you complete a closed geometric shape (like a square or triangle) on the ground, a ritual triggers within that area, obliterating everything inside.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Gameplay Impact:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> It becomes a game of "Snake" mixed with a survivors-like. You are constantly trying to pathfind around enemies to close your shapes without getting trapped.</t>
-    </r>
-  </si>
-  <si>
-    <t>3. Magnetic North</t>
-  </si>
-  <si>
-    <t>All XP gems and items are magnetic. If you move too fast, they trail behind you, forming a massive "tail." If enemies touch the tail, they absorb the XP and evolve into Elites.</t>
-  </si>
-  <si>
-    <t>4. Auction House (Economy Mode)</t>
-  </si>
-  <si>
-    <t>Experience points (XP) are replaced with a currency that fluctuates in value.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Every 3 minutes, the game pauses for a "Blind Auction."</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Powerful items are put up for bid against "AI Rivals" who are also in the map with you. Do you spend all your gold on one Tier-5 weapon now, or save up for the endgame?</t>
-    </r>
-  </si>
-  <si>
-    <t>5. Temporal Echoes (The Time-Loop Mode)</t>
-  </si>
-  <si>
-    <t>The run is divided into short 2-minute loops that stack on top of each other.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> When the 2-minute timer hits zero, you are sent back to the start. However, a "Ghost Echo" of your previous run is now playing alongside you, performing the exact movements and shots you did in the last loop.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> By the 10th loop, there are 10 versions of you on screen. The enemy count scales exponentially to compensate.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Gameplay Impact:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You have to plan your movements in early loops to "cover" yourself for future loops (e.g., "In Loop 1, I'll clear the left side so that in Loop 5, my past self is protecting my flank").</t>
-    </r>
-  </si>
-  <si>
-    <t>6. Shifting Biomes (The Maze Runner)</t>
-  </si>
-  <si>
-    <t>The map is a grid of rooms that physically shift and rearrange every 60 seconds.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You might be in an open field one moment and a narrow corridor the next.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You can see the "next layout" on a minimap. You must position yourself so you don't get crushed by a wall or trapped in a room full of Elites when the shift happens.</t>
-    </r>
-  </si>
-  <si>
-    <t>7. Roulette Weapons</t>
-  </si>
-  <si>
-    <t>Every time you reload or fire X shots, your weapon randomly swaps to a different one in your inventory. You have to build for "generalist" buffs rather than specific weapon synergies.</t>
-  </si>
-  <si>
-    <t>8. The Bodyguard (VIP Escort)</t>
-  </si>
-  <si>
-    <t>You are invincible, but you are protecting a "Client" who is very fragile.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> The Client has terrible AI—they wander toward shiny objects and run away from you if you get too close.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Your weapons aren't just for killing; they are for </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>crowd control</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>. You use knockback and walls to "funnel" the Client toward the exit.</t>
-    </r>
-  </si>
-  <si>
-    <t>10. Shared Pool (Co-op/Versus)</t>
-  </si>
-  <si>
-    <t>You and a rival AI share the same upgrade pool. If the AI picks the "Chain Lightning," it's gone from your draft options forever.</t>
-  </si>
-  <si>
-    <t>14. The Slime Trail</t>
-  </si>
-  <si>
-    <t>You leave a trail of "acid" or "slow" behind you.</t>
-  </si>
-  <si>
-    <t>9. The Shadow (Stalker Mode)</t>
-  </si>
-  <si>
-    <t>An invincible, slow-moving "Shadow" of the player follows you at all times.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> It copies your current build. If you have "Chain Lightning," the Shadow also emits "Chain Lightning."</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> If it touches you, the run ends. You have to balance making yourself powerful enough to kill enemies, but not so powerful that your Shadow becomes impossible to kite.</t>
-    </r>
-  </si>
-  <si>
-    <t>11. Gravity Well</t>
-  </si>
-  <si>
-    <t>The center of the map has a massive gravitational pull.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> All projectiles, enemies, and XP gems curve toward the center.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You can use the gravity to "slingshot" your shots around corners, but staying near the edges makes you move slower as you fight the pull.</t>
-    </r>
-  </si>
-  <si>
-    <t>12. The Architect (Tower Defense)</t>
-  </si>
-  <si>
-    <t>You cannot move. Instead, you click to place traps and turrets.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You have a limited "Energy" pool that refills when enemies die.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You can "possess" one of your turrets for 10 seconds to fire it manually with increased damage.</t>
-    </r>
-  </si>
-  <si>
-    <t>13. Blood Magic</t>
-  </si>
-  <si>
-    <t>You don't have a mana or cooldown system. Everything costs health.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Your primary way to heal is by standing in the "blood splatter" left by defeated enemies.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> The more health you lose, the higher your damage multiplier becomes, encouraging a high-risk "glass cannon" playstyle.</t>
-    </r>
-  </si>
-  <si>
-    <t>15. Minimalist</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">You can only have </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>one</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> weapon and </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>one</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> passive buff at a time.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Every time you level up, you </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>must</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> replace your current item with a new one.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Items scale aggressively. A Level 10 "Basic Pistol" might be stronger than a Level 1 "God Slayer Sword," forcing you to decide when to break your synergy for raw power.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>16. Nano-Swarm:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Instead of a character, you play as a cloud of nanites. You "attack" by overlapping with enemies, but your "health" is the literal size of your swarm.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>17. Darkness Visible:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> The screen is pitch black except for a small radius around you. Enemies only become visible when they are hit by your "radar" pulse or enter your light circle.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>18. Floor is Lava:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You can only stand on "safe tiles" that disappear after 5 seconds. You must constantly move to new platforms while fighting the horde.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>19. Recoil Propulsion:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You have no movement keys. The only way to move is by using the recoil of your weapons to push yourself in the opposite direction.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>20. Boss Rush:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> There are no "trash mobs." Every 30 seconds, a mini-boss spawns. You are constantly fighting 3–4 bosses at once with unique mechanics.</t>
-    </r>
-  </si>
-  <si>
-    <t>21. The Pacifist</t>
-  </si>
-  <si>
-    <t>You cannot deal damage directly.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You have an "Aura of Conversion." Enemies that stay inside your radius for 3 seconds become your allies.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You have to keep your "converted" army alive. If your army dies, you have no way to defend yourself while you "recruit" more.</t>
-    </r>
-  </si>
-  <si>
-    <t>22. Rhythm Heaven (Beat-Based)</t>
-  </si>
-  <si>
-    <t>Your weapons only fire on the beat of the background music.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Perfect timing increases your damage and fire rate.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Missing the beat cause your weapon to "jam" for 2 seconds, leaving you vulnerable.</t>
-    </r>
-  </si>
-  <si>
-    <t>23. The Alchemist (Crafting Mode)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">You don't get weapons from leveling up. You get </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Elements</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (Fire, Water, Iron, Glass).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You must manually combine elements in a crafting menu to create spells (e.g., Fire + Glass = Flaming Shards).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Recipes change every run. You have to spend the first 5 minutes "experimenting" to find the most powerful combinations for that specific run.</t>
-    </r>
-  </si>
-  <si>
-    <t>24. Size Matters</t>
-  </si>
-  <si>
-    <t>Every time you kill an enemy, you grow 1% larger.</t>
-  </si>
-  <si>
-    <r>
-      <t>The Hook:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Being larger increases your health and reach.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>The Twist:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> As you grow, you become a bigger target, move slower, and eventually, you can't fit through narrow gaps in the map, forcing you to stay in open areas.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>25. The Curator:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Instead of a standard skill tree, you unlock "Exhibit Halls" in a museum. Each hall you fill with "Artifacts" (rare drops from bosses) provides permanent stat boosts to specific modes.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>26. Mode Fusion:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Once you beat any two modes, you can "Fuse" them for a Nightmare Run (e.g., </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>The Shadow</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> + </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Floor is Lava</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>27. The Stock Market:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> You can "invest" your meta-currency into different weapon manufacturers. If players globally use the "Shotgun" more this week, the "Shotgun Company" stock goes up, granting you better starting bonuses for those weapons.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>28. Community Challenges:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Every weekend, the developer picks a specific "Seed" and "Mode Combination." Everyone competes on a global leaderboard for a unique cosmetic skin.</t>
-    </r>
-  </si>
-  <si>
-    <t>Core Game Modes</t>
-  </si>
-  <si>
-    <t>Unique Combat &amp; Movement Mechanics</t>
-  </si>
-  <si>
-    <t>Advanced Interaction Modes</t>
-  </si>
-  <si>
-    <t>Meta-Progression &amp; Hub Features</t>
-  </si>
-  <si>
     <t>Psammomancer</t>
   </si>
   <si>
@@ -1730,13 +872,82 @@
   </si>
   <si>
     <t>GravityWell</t>
+  </si>
+  <si>
+    <t>Infect Enemies and that hurts nearby enemies</t>
+  </si>
+  <si>
+    <t>Characters</t>
+  </si>
+  <si>
+    <t>Sigil Architect – The Character drops a trail behind them, and if they enclose the trail, the trail and all enemies within die/take damage</t>
+  </si>
+  <si>
+    <t>Parasite Enemies – Enemies can absorb  XP Gems and evolve into Elites.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auction House – Every 3 minutes, the game pauses for a "Blind Auction." Powerful items are put up for bid against "AI Rivals" who are also in the map with you. </t>
+  </si>
+  <si>
+    <t>Temporal Echoes (The Time-Loop Mode) – The run is divided into short 2-minute loops that stack on top of each other. When the 2-minute timer hits zero, you are sent back to the start. However, a "Ghost Echo" of your previous run is now playing alongside you, performing the exact movements and shots you did in the last loop.</t>
+  </si>
+  <si>
+    <t>Shifting Biomes – The map is a grid of rooms that physically shift and rearrange every 60 seconds.</t>
+  </si>
+  <si>
+    <t>Roulette Weapons – Every 2 minutes, your weapons randomly swaps to different ones</t>
+  </si>
+  <si>
+    <t>The Bodyguard (VIP Escort) – You are invincible, but you are protecting a "Client" who is very fragile.</t>
+  </si>
+  <si>
+    <t>The Shadow – AI with your build spawns every 5 minutes. You must defeat them or lose</t>
+  </si>
+  <si>
+    <t>Shared Pool (Co-op/Versus) – You and a rival AI share the same upgrade pool. If the AI picks the "Chain Lightning," it's gone from your draft options forever.</t>
+  </si>
+  <si>
+    <t>Shared Pool (Co-op/Versus) – You and a rival PVP Player share the same upgrade pool. If the AI picks the "Chain Lightning," it's gone from your draft options forever.</t>
+  </si>
+  <si>
+    <t>Through The Looking Glass – PVP, one player spawns the waves of enemies from a budget, and the other plays the game normally</t>
+  </si>
+  <si>
+    <t>Gravity Well– The center of the map has a massive gravitational pull.</t>
+  </si>
+  <si>
+    <t>The Architect (Tower Defense)</t>
+  </si>
+  <si>
+    <t>lower health = higher damage</t>
+  </si>
+  <si>
+    <t>The Slime Trail – You leave a trail of "acid"  behind you.</t>
+  </si>
+  <si>
+    <t>Minimalist – You can only have one weapon and one passive buff at a time. Every time you level up, you must replace your current item with a new one.</t>
+  </si>
+  <si>
+    <t>Floor is Lava– You can only stand on "safe tiles" that disappear after 5 seconds. You must constantly move to new platforms while fighting the horde.</t>
+  </si>
+  <si>
+    <t>Boss Rush – Every 10 seconds, a mini-boss spawns. Every minute a boss spawns.</t>
+  </si>
+  <si>
+    <t>The Pacifist(Character) You cannot deal damage directly. You have an "Aura of Conversion." Enemies that stay inside your radius for 3 seconds become your allies.</t>
+  </si>
+  <si>
+    <t>Mode Fusion– Once you beat any two modes, you can "Fuse" them for a Nightmare Run (e.g., The Shadow + Floor is Lava).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Community Challenges– Every weekend, the developer picks a specific "Seed" and "Mode Combination." Everyone competes on a global leaderboard </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1766,40 +977,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13.5"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1846,7 +1023,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1860,19 +1037,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2201,12 +1372,12 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>356</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>355</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -2877,7 +2048,7 @@
         <v>182</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>357</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2890,7 +2061,7 @@
       <c r="C2" t="s">
         <v>184</v>
       </c>
-      <c r="D2" s="11"/>
+      <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -2902,7 +2073,7 @@
       <c r="C3" t="s">
         <v>186</v>
       </c>
-      <c r="D3" s="11"/>
+      <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -2914,7 +2085,7 @@
       <c r="C4" t="s">
         <v>133</v>
       </c>
-      <c r="D4" s="11"/>
+      <c r="D4" s="7"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -2926,7 +2097,7 @@
       <c r="C5" t="s">
         <v>135</v>
       </c>
-      <c r="D5" s="11"/>
+      <c r="D5" s="7"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -2938,7 +2109,7 @@
       <c r="C6" t="s">
         <v>190</v>
       </c>
-      <c r="D6" s="11"/>
+      <c r="D6" s="7"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -2961,7 +2132,7 @@
       <c r="C8" t="s">
         <v>193</v>
       </c>
-      <c r="D8" s="11"/>
+      <c r="D8" s="7"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -3017,7 +2188,7 @@
       <c r="C13" t="s">
         <v>256</v>
       </c>
-      <c r="D13" s="11"/>
+      <c r="D13" s="7"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -3073,7 +2244,7 @@
       <c r="C18" t="s">
         <v>212</v>
       </c>
-      <c r="D18" s="11"/>
+      <c r="D18" s="7"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
@@ -3129,7 +2300,7 @@
       <c r="C23" t="s">
         <v>222</v>
       </c>
-      <c r="D23" s="11"/>
+      <c r="D23" s="7"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
@@ -3172,7 +2343,7 @@
         <v>226</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>354</v>
+        <v>271</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -3185,7 +2356,7 @@
       <c r="C28" t="s">
         <v>257</v>
       </c>
-      <c r="D28" s="11"/>
+      <c r="D28" s="7"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
@@ -3208,7 +2379,7 @@
       <c r="C30" t="s">
         <v>232</v>
       </c>
-      <c r="D30" s="11"/>
+      <c r="D30" s="7"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
@@ -3220,7 +2391,7 @@
       <c r="C31" t="s">
         <v>234</v>
       </c>
-      <c r="D31" s="11"/>
+      <c r="D31" s="7"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
@@ -3276,7 +2447,7 @@
       <c r="C36" t="s">
         <v>258</v>
       </c>
-      <c r="D36" s="11"/>
+      <c r="D36" s="7"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
@@ -3365,7 +2536,7 @@
       <c r="C44" t="s">
         <v>166</v>
       </c>
-      <c r="D44" s="11"/>
+      <c r="D44" s="7"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
@@ -3377,72 +2548,72 @@
       <c r="C45" t="s">
         <v>169</v>
       </c>
-      <c r="D45" s="11"/>
+      <c r="D45" s="7"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>342</v>
+        <v>259</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>343</v>
+        <v>260</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>344</v>
+        <v>261</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>345</v>
+        <v>262</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>347</v>
+        <v>264</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>346</v>
+        <v>263</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>348</v>
+        <v>265</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>350</v>
+        <v>267</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>351</v>
+        <v>268</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>349</v>
+        <v>266</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>352</v>
+        <v>269</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>353</v>
+        <v>270</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>358</v>
+        <v>275</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>359</v>
+        <v>276</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>360</v>
+        <v>277</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>361</v>
+        <v>278</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>362</v>
+        <v>279</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>363</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -3453,422 +2624,121 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC19137E-1A1C-4137-828B-A034EA426793}">
-  <dimension ref="A1:A86"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="80.21875" style="9" customWidth="1"/>
+    <col min="2" max="2" width="38.77734375" style="9" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A26" s="10" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A28" s="10" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" s="7" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A30" s="9" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A32" s="10" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="7" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A36" s="10" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" s="7" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A38" s="10" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" s="7" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" s="9" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A41" s="9" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A42" s="10" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" s="7" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="9" t="s">
         <v>303</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" s="9" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A46" s="10" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="7" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="9" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A50" s="10" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="7" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A52" s="10" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="7" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" s="9" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" s="9" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="8" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" s="9" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A59" s="9" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" s="9" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A61" s="9" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A62" s="9" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A64" s="8" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A65" s="10" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A66" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A67" s="9" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A68" s="9" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A69" s="10" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A70" s="7" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A71" s="9" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A72" s="9" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A73" s="10" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A74" s="7" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A75" s="9" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A76" s="9" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A77" s="10" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A78" s="7" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A79" s="9" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A80" s="9" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A82" s="8" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A83" s="9" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A84" s="9" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A85" s="9" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A86" s="9" t="s">
-        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>